<commit_message>
Clean MAPR artifact package: remove SOICT + anonymize reviewer inputs
</commit_message>
<xml_diff>
--- a/output/mapr_analysis_tables.xlsx
+++ b/output/mapr_analysis_tables.xlsx
@@ -1693,7 +1693,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>3443401</t>
+          <t>S0010</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -1730,7 +1730,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>3443661</t>
+          <t>S0059</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -1767,7 +1767,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>3443421</t>
+          <t>S0014</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -1804,7 +1804,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>3443506</t>
+          <t>S0030</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -1841,7 +1841,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>3443511</t>
+          <t>S0031</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -1878,7 +1878,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>3443551</t>
+          <t>S0038</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -1915,7 +1915,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>3443676</t>
+          <t>S0062</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -1952,7 +1952,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>3443736</t>
+          <t>S0074</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -1989,7 +1989,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>3443991</t>
+          <t>S0122</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -2026,7 +2026,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>3443386</t>
+          <t>S0007</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -2063,7 +2063,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>3443396</t>
+          <t>S0009</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -2100,7 +2100,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>3443561</t>
+          <t>S0039</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -2137,7 +2137,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>3443636</t>
+          <t>S0054</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -2174,7 +2174,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>3443656</t>
+          <t>S0058</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -2211,7 +2211,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>3443671</t>
+          <t>S0061</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -2248,7 +2248,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>3443691</t>
+          <t>S0065</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -2285,7 +2285,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>3443731</t>
+          <t>S0073</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -2322,7 +2322,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>3443891</t>
+          <t>S0103</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -2359,7 +2359,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>3443701</t>
+          <t>S0067</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -2396,7 +2396,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>3443946</t>
+          <t>S0113</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -2433,7 +2433,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>3443621</t>
+          <t>S0051</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -2470,7 +2470,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>3444061</t>
+          <t>S0136</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -2507,7 +2507,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>3443371</t>
+          <t>S0004</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -2544,7 +2544,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>3443416</t>
+          <t>S0013</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -2581,7 +2581,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>3443426</t>
+          <t>S0015</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -2618,7 +2618,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>3443471</t>
+          <t>S0024</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -2655,7 +2655,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>3443486</t>
+          <t>S0026</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -2692,7 +2692,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>3443516</t>
+          <t>S0032</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -2729,7 +2729,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>3443641</t>
+          <t>S0055</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -2766,7 +2766,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>3443926</t>
+          <t>S0109</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -2874,7 +2874,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>3810590</t>
+          <t>S0251</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -2911,7 +2911,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>3735320</t>
+          <t>S0163</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -2948,7 +2948,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>3810470</t>
+          <t>S0229</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -2985,7 +2985,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>3735345</t>
+          <t>S0167</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -3022,7 +3022,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>3735200</t>
+          <t>S0141</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -3059,7 +3059,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>3735525</t>
+          <t>S0198</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -3096,7 +3096,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>3810515</t>
+          <t>S0238</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -3133,7 +3133,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>3810685</t>
+          <t>S0266</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -3170,7 +3170,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>3735215</t>
+          <t>S0144</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -3207,7 +3207,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>3735285</t>
+          <t>S0156</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -3244,7 +3244,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>3735290</t>
+          <t>S0157</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -3281,7 +3281,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>3735355</t>
+          <t>S0169</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -3318,7 +3318,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>3735530</t>
+          <t>S0199</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -3355,7 +3355,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>3810355</t>
+          <t>S0207</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -3392,7 +3392,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>3810380</t>
+          <t>S0212</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -3429,7 +3429,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>3810390</t>
+          <t>S0213</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -3466,7 +3466,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>3810555</t>
+          <t>S0245</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -3503,7 +3503,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>3810575</t>
+          <t>S0248</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -3540,7 +3540,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>3810675</t>
+          <t>S0264</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -3577,7 +3577,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>3735305</t>
+          <t>S0160</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -3614,7 +3614,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>3735490</t>
+          <t>S0193</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -3651,7 +3651,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>3810365</t>
+          <t>S0209</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -3688,7 +3688,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>3735280</t>
+          <t>S0155</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -3725,7 +3725,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>3810430</t>
+          <t>S0221</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -3762,7 +3762,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>3810450</t>
+          <t>S0225</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -3799,7 +3799,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>3810465</t>
+          <t>S0228</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -3836,7 +3836,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>3810565</t>
+          <t>S0247</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -3873,7 +3873,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>3810585</t>
+          <t>S0250</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -3910,7 +3910,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>3810455</t>
+          <t>S0226</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -3947,7 +3947,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>3735430</t>
+          <t>S0181</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -4055,7 +4055,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>3875900</t>
+          <t>S0363</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -4092,7 +4092,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>3875785</t>
+          <t>S0344</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -4129,7 +4129,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>3875735</t>
+          <t>S0337</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -4166,7 +4166,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>3873515</t>
+          <t>S0305</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -4203,7 +4203,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>3873580</t>
+          <t>S0317</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -4240,7 +4240,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>3873645</t>
+          <t>S0329</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -4277,7 +4277,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>3876055</t>
+          <t>S0387</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -4314,7 +4314,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>3873655</t>
+          <t>S0331</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -4351,7 +4351,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>3873360</t>
+          <t>S0278</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -4388,7 +4388,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>3875905</t>
+          <t>S0364</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -4425,7 +4425,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>3875915</t>
+          <t>S0366</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -4462,7 +4462,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>3873330</t>
+          <t>S0272</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -4499,7 +4499,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>3873375</t>
+          <t>S0281</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -4536,7 +4536,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>3873395</t>
+          <t>S0284</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -4573,7 +4573,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>3873495</t>
+          <t>S0302</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -4610,7 +4610,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>3873640</t>
+          <t>S0328</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -4647,7 +4647,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>3873345</t>
+          <t>S0275</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -4684,7 +4684,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>3873370</t>
+          <t>S0280</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -4721,7 +4721,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>3873540</t>
+          <t>S0310</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -4758,7 +4758,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>3873620</t>
+          <t>S0325</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -4795,7 +4795,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>3875860</t>
+          <t>S0357</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -4832,7 +4832,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>3876050</t>
+          <t>S0386</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -4869,7 +4869,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>3873380</t>
+          <t>S0282</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -4906,7 +4906,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>3873410</t>
+          <t>S0287</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -4943,7 +4943,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>3873415</t>
+          <t>S0288</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -4980,7 +4980,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>3873445</t>
+          <t>S0293</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -5017,7 +5017,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>3873470</t>
+          <t>S0298</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -5054,7 +5054,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>3873490</t>
+          <t>S0301</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -5091,7 +5091,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>3873660</t>
+          <t>S0332</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -5128,7 +5128,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>3876045</t>
+          <t>S0385</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -5236,7 +5236,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>4052097</t>
+          <t>S0391</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -5273,7 +5273,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>4052352</t>
+          <t>S0438</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -5310,7 +5310,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>4112597</t>
+          <t>S0459</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -5347,7 +5347,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>4112707</t>
+          <t>S0478</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -5384,7 +5384,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>4112722</t>
+          <t>S0481</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -5421,7 +5421,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>4112752</t>
+          <t>S0487</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -5458,7 +5458,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>4052167</t>
+          <t>S0404</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -5495,7 +5495,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>4052137</t>
+          <t>S0398</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -5532,7 +5532,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>4052287</t>
+          <t>S0426</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -5569,7 +5569,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>4052302</t>
+          <t>S0429</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -5606,7 +5606,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>4052332</t>
+          <t>S0434</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -5643,7 +5643,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>4052337</t>
+          <t>S0435</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -5680,7 +5680,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>4052342</t>
+          <t>S0436</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -5717,7 +5717,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>4052417</t>
+          <t>S0450</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -5754,7 +5754,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>4052427</t>
+          <t>S0452</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -5791,7 +5791,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>4052432</t>
+          <t>S0453</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -5828,7 +5828,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>4112617</t>
+          <t>S0463</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -5865,7 +5865,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>4112692</t>
+          <t>S0475</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -5902,7 +5902,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>4112702</t>
+          <t>S0477</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -5939,7 +5939,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>4112747</t>
+          <t>S0486</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -5976,7 +5976,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>4112842</t>
+          <t>S0505</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -6013,7 +6013,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>4052212</t>
+          <t>S0411</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -6050,7 +6050,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>4052117</t>
+          <t>S0394</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -6087,7 +6087,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>4112797</t>
+          <t>S0496</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -6124,7 +6124,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>4112802</t>
+          <t>S0497</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -6161,7 +6161,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>4052142</t>
+          <t>S0399</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -6198,7 +6198,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>4052222</t>
+          <t>S0413</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -6235,7 +6235,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>4112812</t>
+          <t>S0499</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -6272,7 +6272,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>4052237</t>
+          <t>S0416</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -6309,7 +6309,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>4052262</t>
+          <t>S0421</t>
         </is>
       </c>
       <c r="B31" t="n">

</xml_diff>